<commit_message>
add decision boundary matrix figure, resized asset, and improvement data spreadsheet
</commit_message>
<xml_diff>
--- a/scratch/figures/Improvement_Figures.xlsx
+++ b/scratch/figures/Improvement_Figures.xlsx
@@ -156,7 +156,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10477500" cy="6429375"/>
+    <ext cx="10477500" cy="6715125"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -639,6 +639,8 @@
     <row r="55" ht="15" customHeight="1"/>
     <row r="56" ht="15" customHeight="1"/>
     <row r="57" ht="15" customHeight="1"/>
+    <row r="58" ht="15" customHeight="1"/>
+    <row r="59" ht="15" customHeight="1"/>
     <row r="85">
       <c r="B85" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add agglomerative clustering pipeline and figure generation scripts with common utilities
</commit_message>
<xml_diff>
--- a/scratch/figures/Improvement_Figures.xlsx
+++ b/scratch/figures/Improvement_Figures.xlsx
@@ -156,7 +156,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10477500" cy="6715125"/>
+    <ext cx="10477500" cy="6781800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -181,7 +181,7 @@
       <row>87</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10477500" cy="3752850"/>
+    <ext cx="10477500" cy="3924300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -206,7 +206,7 @@
       <row>167</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10477500" cy="8715375"/>
+    <ext cx="10477500" cy="8848725"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -231,7 +231,7 @@
       <row>247</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10477500" cy="6305550"/>
+    <ext cx="10477500" cy="6362700"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -571,7 +571,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Generated from the Selected_Data_RFE and Morris_Sensitivity(RFE) sheets. Binary classification target = Execution Efficiency Class (0 = Best, &gt;0 = Other grouped).</t>
+          <t>Generated from the data_after_chi2 and Morris_Sensitivity(Chi2) sheets. Binary classification target = Execution Efficiency Class (0 = Best, &gt;0 = Other grouped).</t>
         </is>
       </c>
     </row>
@@ -686,6 +686,7 @@
     <row r="116" ht="15" customHeight="1"/>
     <row r="117" ht="15" customHeight="1"/>
     <row r="118" ht="15" customHeight="1"/>
+    <row r="119" ht="15" customHeight="1"/>
     <row r="165">
       <c r="B165" s="3" t="inlineStr">
         <is>

</xml_diff>